<commit_message>
Add English-first multilingual interface
</commit_message>
<xml_diff>
--- a/examples/import/schools.xlsx
+++ b/examples/import/schools.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Школы (учебные данные)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Описание" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Schools (sample data)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Description" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,22 +436,22 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Код школы</t>
+          <t>School ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Тип школы</t>
+          <t>School type</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Учащиеся</t>
+          <t>Students</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Учителя</t>
+          <t>Teachers</t>
         </is>
       </c>
     </row>
@@ -463,7 +463,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Городская</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -481,7 +481,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Сельская</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -499,7 +499,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Лицей</t>
+          <t>Lyceum</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -517,7 +517,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Городская</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -535,7 +535,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Сельская</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -553,7 +553,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Лицей</t>
+          <t>Lyceum</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Городская</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -589,7 +589,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Сельская</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -607,7 +607,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Лицей</t>
+          <t>Lyceum</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Городская</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -643,10 +643,9 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Сельская</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>Rural</t>
+        </is>
+      </c>
       <c r="D12" t="n">
         <v>14</v>
       </c>
@@ -659,7 +658,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Лицей</t>
+          <t>Lyceum</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -677,7 +676,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Городская</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -695,7 +694,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Сельская</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -713,7 +712,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Лицей</t>
+          <t>Lyceum</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -731,7 +730,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Городская</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -749,7 +748,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Сельская</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -767,7 +766,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Лицей</t>
+          <t>Lyceum</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -775,7 +774,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -787,7 +786,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Городская</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -805,7 +804,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Сельская</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -823,7 +822,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Лицей</t>
+          <t>Lyceum</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -841,7 +840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Городская</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -859,7 +858,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Сельская</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -877,7 +876,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Лицей</t>
+          <t>Lyceum</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -904,21 +903,21 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Учебный набор — вымышленные школы</t>
+          <t>Sample dataset — fictional schools</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Одна строка = одна школа; период = 2025 год.</t>
+          <t>One row = one fictional school; period = 2025.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Для проверки импорта. Не официальная статистика.</t>
+          <t>Import example. Not official statistics.</t>
         </is>
       </c>
     </row>

</xml_diff>